<commit_message>
EXP-014: break out master/sub tokens into input vs output
Adds per-role input/output breakdown to the master/sub token split. Each
agent's master/sub share is measured (two-model validation); the input/output
split within each role applies the measured per-role in:out ratio from the
two-model token_count by model+type (master 88:12, sub 61:39). Per-agent §4
gains master/sub input+output rows; xlsx adds 4 breakdown columns.
</commit_message>
<xml_diff>
--- a/agent_summaries/MASTER_SUMMARY.xlsx
+++ b/agent_summaries/MASTER_SUMMARY.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SKU matrix'!$A$1:$S$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SKU matrix'!$A$1:$W$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:W14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -473,6 +473,10 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,60 +517,80 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Master input</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Master output</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-agent input</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-agent output</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Model calls</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>vCPU-seconds</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>GiB-seconds</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Session events</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Mem-gen tokens</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Memories retrieved</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Firestore writes</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Firestore reads</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>RAG queries</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Web grounding</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Imagen images</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>$/interaction</t>
         </is>
@@ -596,40 +620,52 @@
       <c r="G2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="4" t="n">
+        <v>6368.8333</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>692.5333000000001</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="5" t="n">
         <v>7.5083</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="M2" s="5" t="n">
         <v>20.86194231014962</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="N2" s="5" t="n">
         <v>38.80402965164957</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="O2" s="5" t="n">
         <v>15.0167</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="P2" s="4" t="n">
         <v>2485.783333333333</v>
       </c>
-      <c r="M2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6" t="n">
+      <c r="Q2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="6" t="n">
         <v>0.03333333333333333</v>
       </c>
-      <c r="O2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="6" t="n">
+      <c r="S2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" s="6" t="n">
         <v>2.15</v>
       </c>
-      <c r="Q2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" s="7" t="n">
+      <c r="U2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" s="7" t="n">
         <v>0.01390041782237551</v>
       </c>
     </row>
@@ -657,40 +693,52 @@
       <c r="G3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="4" t="n">
+        <v>20106.6186</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>1484.6949</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="5" t="n">
         <v>13.9576</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="M3" s="5" t="n">
         <v>25.29153067805368</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="N3" s="5" t="n">
         <v>46.79568050274576</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="O3" s="5" t="n">
         <v>27.9492</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="P3" s="4" t="n">
         <v>2548.906779661017</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="Q3" s="6" t="n">
         <v>0.6694915254237288</v>
       </c>
-      <c r="N3" s="6" t="n">
+      <c r="R3" s="6" t="n">
         <v>1.423728813559322</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="S3" s="6" t="n">
         <v>1.228813559322034</v>
       </c>
-      <c r="P3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="7" t="n">
+      <c r="T3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="7" t="n">
         <v>0.02322548602823488</v>
       </c>
     </row>
@@ -718,40 +766,52 @@
       <c r="G4" s="4" t="n">
         <v>3855.844900000001</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="4" t="n">
+        <v>30513.52715685331</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>8209.629315345892</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>2071.372843146695</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>2529.570684654109</v>
+      </c>
+      <c r="L4" s="5" t="n">
         <v>7.7848</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="M4" s="5" t="n">
         <v>171.2293533162262</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="N4" s="5" t="n">
         <v>200.603827065459</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="O4" s="5" t="n">
         <v>15.5696</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="P4" s="4" t="n">
         <v>7998.772151898735</v>
       </c>
-      <c r="M4" s="6" t="n">
+      <c r="Q4" s="6" t="n">
         <v>0.379746835443038</v>
       </c>
-      <c r="N4" s="6" t="n">
+      <c r="R4" s="6" t="n">
         <v>1.341772151898734</v>
       </c>
-      <c r="O4" s="6" t="n">
+      <c r="S4" s="6" t="n">
         <v>2.063291139240506</v>
       </c>
-      <c r="P4" s="6" t="n">
+      <c r="T4" s="6" t="n">
         <v>1.177215189873418</v>
       </c>
-      <c r="Q4" s="6" t="n">
+      <c r="U4" s="6" t="n">
         <v>1.620253164556962</v>
       </c>
-      <c r="R4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="7" t="n">
+      <c r="V4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="7" t="n">
         <v>0.08219238927717809</v>
       </c>
     </row>
@@ -779,40 +839,52 @@
       <c r="G5" s="4" t="n">
         <v>129092.6</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="4" t="n">
+        <v>33567.55519077396</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>365.8113818097356</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>115512.236509226</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>5713.771918190265</v>
+      </c>
+      <c r="L5" s="5" t="n">
         <v>18.925</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="M5" s="5" t="n">
         <v>90.55245122597219</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="N5" s="5" t="n">
         <v>100.3361411779296</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="O5" s="5" t="n">
         <v>37.8917</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="P5" s="4" t="n">
         <v>2792.833333333333</v>
       </c>
-      <c r="M5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="N5" s="6" t="n">
+      <c r="R5" s="6" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="S5" s="6" t="n">
         <v>0.6333333333333333</v>
       </c>
-      <c r="P5" s="6" t="n">
+      <c r="T5" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
-      <c r="Q5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="7" t="n">
+      <c r="U5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="7" t="n">
         <v>0.09322426317660537</v>
       </c>
     </row>
@@ -840,40 +912,52 @@
       <c r="G6" s="4" t="n">
         <v>5844.150600000001</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="4" t="n">
+        <v>20188.60869847577</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>5846.493636244672</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>3016.991301524224</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>3965.706363755328</v>
+      </c>
+      <c r="L6" s="5" t="n">
         <v>3.4875</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="M6" s="5" t="n">
         <v>135.6170507841798</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="N6" s="5" t="n">
         <v>174.0941383997125</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="O6" s="5" t="n">
         <v>7.225</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="P6" s="4" t="n">
         <v>3150.6875</v>
       </c>
-      <c r="M6" s="6" t="n">
+      <c r="Q6" s="6" t="n">
         <v>0.55</v>
       </c>
-      <c r="N6" s="6" t="n">
+      <c r="R6" s="6" t="n">
         <v>0.025</v>
       </c>
-      <c r="O6" s="6" t="n">
+      <c r="S6" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="P6" s="6" t="n">
+      <c r="T6" s="6" t="n">
         <v>0.2625</v>
       </c>
-      <c r="Q6" s="6" t="n">
+      <c r="U6" s="6" t="n">
         <v>0.9</v>
       </c>
-      <c r="R6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="7" t="n">
+      <c r="V6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="7" t="n">
         <v>0.05947523090556715</v>
       </c>
     </row>
@@ -901,40 +985,52 @@
       <c r="G7" s="4" t="n">
         <v>1372.9392</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="4" t="n">
+        <v>3681.064591925444</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>555.1221854470177</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>825.5354080745565</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>565.0778145529823</v>
+      </c>
+      <c r="L7" s="5" t="n">
         <v>2.975</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="M7" s="5" t="n">
         <v>66.4738146469108</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="N7" s="5" t="n">
         <v>85.22285866436781</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="O7" s="5" t="n">
         <v>6.05</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="P7" s="4" t="n">
         <v>2479.725</v>
       </c>
-      <c r="M7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="6" t="n">
+      <c r="Q7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="6" t="n">
         <v>0.0375</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="S7" s="6" t="n">
         <v>0.5625</v>
       </c>
-      <c r="P7" s="6" t="n">
+      <c r="T7" s="6" t="n">
         <v>0.3375</v>
       </c>
-      <c r="Q7" s="6" t="n">
+      <c r="U7" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="R7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="7" t="n">
+      <c r="V7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="7" t="n">
         <v>0.02011496261319722</v>
       </c>
     </row>
@@ -962,40 +1058,52 @@
       <c r="G8" s="4" t="n">
         <v>1061.8852</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="4" t="n">
+        <v>9761.461877912679</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>3231.761408322597</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>542.0381220873197</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>814.5385916774035</v>
+      </c>
+      <c r="L8" s="5" t="n">
         <v>3.7</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="M8" s="5" t="n">
         <v>187.9178019633661</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="N8" s="5" t="n">
         <v>231.3129107875827</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="O8" s="5" t="n">
         <v>7.6125</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="P8" s="4" t="n">
         <v>2762.25</v>
       </c>
-      <c r="M8" s="6" t="n">
+      <c r="Q8" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="N8" s="6" t="n">
+      <c r="R8" s="6" t="n">
         <v>0.05</v>
       </c>
-      <c r="O8" s="6" t="n">
+      <c r="S8" s="6" t="n">
         <v>1.0125</v>
       </c>
-      <c r="P8" s="6" t="n">
+      <c r="T8" s="6" t="n">
         <v>1.7</v>
       </c>
-      <c r="Q8" s="6" t="n">
+      <c r="U8" s="6" t="n">
         <v>0.525</v>
       </c>
-      <c r="R8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="7" t="n">
+      <c r="V8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="7" t="n">
         <v>0.03390983380696357</v>
       </c>
     </row>
@@ -1023,40 +1131,52 @@
       <c r="G9" s="4" t="n">
         <v>4813.0761</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="4" t="n">
+        <v>8865.463371117343</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>2390.447682368085</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>2479.636628882657</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>3034.752317631915</v>
+      </c>
+      <c r="L9" s="5" t="n">
         <v>4.8</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="M9" s="5" t="n">
         <v>101.3156201557057</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="N9" s="5" t="n">
         <v>137.7952636383738</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="O9" s="5" t="n">
         <v>11.125</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="P9" s="4" t="n">
         <v>4603.375</v>
       </c>
-      <c r="M9" s="6" t="n">
+      <c r="Q9" s="6" t="n">
         <v>0.3125</v>
       </c>
-      <c r="N9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="6" t="n">
+      <c r="R9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="P9" s="6" t="n">
+      <c r="T9" s="6" t="n">
         <v>0.8</v>
       </c>
-      <c r="Q9" s="6" t="n">
+      <c r="U9" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="R9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="7" t="n">
+      <c r="V9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="7" t="n">
         <v>0.06382839242043145</v>
       </c>
     </row>
@@ -1078,40 +1198,44 @@
       </c>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="5" t="n">
         <v>17.1714</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="M10" s="5" t="n">
         <v>322.7169288552903</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="N10" s="5" t="n">
         <v>328.9131032095976</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="O10" s="5" t="n">
         <v>31.6286</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="P10" s="4" t="n">
         <v>4191.028571428571</v>
       </c>
-      <c r="M10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="Q10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="R10" s="3" t="n">
+      <c r="R10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="S10" s="7" t="n">
+      <c r="W10" s="7" t="n">
         <v>0.09338430905055096</v>
       </c>
     </row>
@@ -1133,40 +1257,44 @@
       </c>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="M11" s="5" t="n">
         <v>104.1182180611634</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="N11" s="5" t="n">
         <v>127.2010318991755</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="O11" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="P11" s="4" t="n">
         <v>2852.657142857143</v>
       </c>
-      <c r="M11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="R11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="7" t="n">
+      <c r="R11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="7" t="n">
         <v>0.01430562267321586</v>
       </c>
     </row>
@@ -1186,40 +1314,44 @@
       </c>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="5" t="n">
         <v>5.75</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="M12" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="N12" s="5" t="n">
         <v>560</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="O12" s="5" t="n">
         <v>11.5</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="P12" s="4" t="n">
         <v>2493</v>
       </c>
-      <c r="M12" s="6" t="n">
+      <c r="Q12" s="6" t="n">
         <v>2.5</v>
       </c>
-      <c r="N12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="7" t="n">
+      <c r="R12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="7" t="n">
         <v>0.0165</v>
       </c>
     </row>
@@ -1241,40 +1373,44 @@
       </c>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="5" t="n">
         <v>2.2857</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="M13" s="5" t="n">
         <v>30.06980230622891</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="N13" s="5" t="n">
         <v>54.58200981646213</v>
       </c>
-      <c r="K13" s="5" t="n">
+      <c r="O13" s="5" t="n">
         <v>4.7714</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="P13" s="4" t="n">
         <v>2357.657142857143</v>
       </c>
-      <c r="M13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="R13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="7" t="n">
+      <c r="R13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="7" t="n">
         <v>0.003525655991319221</v>
       </c>
     </row>
@@ -1296,45 +1432,49 @@
       </c>
       <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
-      <c r="H14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="5" t="n">
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5" t="n">
         <v>12.75356417627951</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="N14" s="5" t="n">
         <v>37.12213692158077</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="O14" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="P14" s="4" t="n">
         <v>2389.885714285714</v>
       </c>
-      <c r="M14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="6" t="n">
-        <v>0</v>
-      </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="R14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="7" t="n">
+      <c r="R14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="7" t="n">
         <v>0.001130142311106089</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S14"/>
+  <autoFilter ref="A1:W14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -1360,7 +1500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1442,134 +1582,146 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Model calls</t>
+          <t>Master/Sub input &amp; output</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Model invocations per interaction. NOT a billing unit (Gemini bills tokens) — a usage driver.</t>
+          <t>The master/sub totals broken into input vs output, via the measured per-role in:out ratio (master 88:12, sub 61:39, from the two-model token_count by model+type). master_in+sub_in = Input tokens; master_out+sub_out = Output tokens.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>vCPU-s / GiB-s</t>
+          <t>Model calls</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Agent Runtime allocation-time, amortized over the window incl. idle. ESTIMATE, not actual instance-hours.</t>
+          <t>Model invocations per interaction. NOT a billing unit (Gemini bills tokens) — a usage driver.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Session events</t>
+          <t>vCPU-s / GiB-s</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Events appended to Sessions. Observed (not metered); excludes session storage GiB-hr.</t>
+          <t>Agent Runtime allocation-time, amortized over the window incl. idle. ESTIMATE, not actual instance-hours.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Mem-gen tokens</t>
+          <t>Session events</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Memory Bank generation tokens (add_session_to_memory). Priced at input rate (proxy); excludes monthly storage.</t>
+          <t>Events appended to Sessions. Observed (not metered); excludes session storage GiB-hr.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Memories retrieved</t>
+          <t>Mem-gen tokens</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Memory Bank memories returned via load_memory. BILLING-ACCURATE ($0.5/1K).</t>
+          <t>Memory Bank generation tokens (add_session_to_memory). Priced at input rate (proxy); excludes monthly storage.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Firestore writes/reads</t>
+          <t>Memories retrieved</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Firestore document ops (save_note/load_note). BILLING-ACCURATE. NOTE: Firestore is not in the GE AP calculator (added as a representative operational DB).</t>
+          <t>Memory Bank memories returned via load_memory. BILLING-ACCURATE ($0.5/1K).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>RAG queries</t>
+          <t>Firestore writes/reads</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Vertex AI Search queries. BILLING-ACCURATE ($1.5/1K); indexed-data storage not captured.</t>
+          <t>Firestore document ops (save_note/load_note). BILLING-ACCURATE. NOTE: Firestore is not in the GE AP calculator (added as a representative operational DB).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Web grounding</t>
+          <t>RAG queries</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Google Search grounded query-turns (web-research AgentTool calls). PROXY/lower bound; billed per grounded prompt ($14/1K).</t>
+          <t>Vertex AI Search queries. BILLING-ACCURATE ($1.5/1K); indexed-data storage not captured.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Imagen images</t>
+          <t>Web grounding</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Images generated (Imagen / gemini-2.5-flash-image). BILLING-ACCURATE (flat-rate estimate).</t>
+          <t>Google Search grounded query-turns (web-research AgentTool calls). PROXY/lower bound; billed per grounded prompt ($14/1K).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
+          <t>Imagen images</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Images generated (Imagen / gemini-2.5-flash-image). BILLING-ACCURATE (flat-rate estimate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
           <t>$/interaction</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Derived cost = Σ(usage × catalog LIST price); incl. Model Armor. REFERENCE ONLY — not billed dollars (no discounts/CUDs).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr"/>
-      <c r="B17" s="10" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr"/>
+      <c r="B18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Uncaptured SKUs</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Apigee, BigQuery, Veo, Maps grounding, Agent Sandbox, Agent Gateway, Cloud Logging/Trace/Monitoring, Agent Evaluation — parked/deferred/pending.</t>
         </is>

</xml_diff>